<commit_message>
Initial commit - RPM calculator
</commit_message>
<xml_diff>
--- a/Backend/data.xlsx
+++ b/Backend/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://torusrobotics-my.sharepoint.com/personal/inventory_torusrobotics_com/Documents/Desktop/vesc-ocr/vesc-ocr/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://torusrobotics-my.sharepoint.com/personal/inventory_torusrobotics_com/Documents/Desktop/vesc-ocr/Backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_61ED52B4D38056381B1A2211595ED87656CD44F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF7501DB-A5BB-43F4-BC46-504AE5800B34}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_61ED52B4D38056381B1A2211595ED87656CD44F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16F3D565-D1F1-47F2-9B7D-AD7A73BB42A0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>id</t>
   </si>
@@ -62,45 +62,6 @@
   </si>
   <si>
     <t>image_url</t>
-  </si>
-  <si>
-    <t>Motor Name</t>
-  </si>
-  <si>
-    <t>Date &amp; Time</t>
-  </si>
-  <si>
-    <t>Power</t>
-  </si>
-  <si>
-    <t>Duty</t>
-  </si>
-  <si>
-    <t>ERPM</t>
-  </si>
-  <si>
-    <t>I Batt</t>
-  </si>
-  <si>
-    <t>I Motor</t>
-  </si>
-  <si>
-    <t>T FET</t>
-  </si>
-  <si>
-    <t>T Motor</t>
-  </si>
-  <si>
-    <t>Volts In</t>
-  </si>
-  <si>
-    <t>Normal ERPM</t>
-  </si>
-  <si>
-    <t>48V RPM</t>
-  </si>
-  <si>
-    <t>Image URL</t>
   </si>
   <si>
     <t>c2</t>
@@ -555,6 +516,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="14" max="14" width="36" customWidth="1"/>
+    <col min="15" max="15" width="29.109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -599,55 +565,29 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>185.5</v>
@@ -677,7 +617,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N2" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -685,10 +625,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D3">
         <v>185.5</v>
@@ -718,7 +658,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N3" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
@@ -726,10 +666,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="D4">
         <v>185.5</v>
@@ -759,7 +699,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N4" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
@@ -767,10 +707,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D5">
         <v>185.5</v>
@@ -800,7 +740,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N5" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
@@ -808,10 +748,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D6">
         <v>185.5</v>
@@ -841,7 +781,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N6" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
@@ -849,10 +789,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <v>185.5</v>
@@ -882,7 +822,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N7" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -890,10 +830,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D8">
         <v>478.7</v>
@@ -923,7 +863,7 @@
         <v>3679.1428571428569</v>
       </c>
       <c r="N8" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
@@ -931,10 +871,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="D9">
         <v>478.7</v>
@@ -964,7 +904,7 @@
         <v>3679.1428571428569</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
@@ -972,10 +912,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D10">
         <v>185.5</v>
@@ -1005,7 +945,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N10" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
@@ -1013,10 +953,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="D11">
         <v>185.5</v>
@@ -1046,7 +986,7 @@
         <v>3722.2857142857142</v>
       </c>
       <c r="N11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>